<commit_message>
Correct SYSPLAN-4237 cases 01/02/03/13 against live DEM Agent evidence
Live check on grs-mac-ssh (tenant 1340, build 54) with DEM Agent actually
running overturned two assumptions: the old in-process m_demMgr/nsDemTaskMgr
was never replaced (still inits at NSClient startup), and the standalone
agent's app-probe traffic is tunneled through NSClient (only the Polaris
event path bypasses it) -- not fully decoupled as the NPLAN note implied.
Raw nsdebuglog.log evidence (line-numbered) added alongside the sysplan.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>NSClient's own startup/init sequence must be the sole trigger for DEM Agent start -- the agent does not auto-start on its own (note Q2b). Live-verified on grs-mac-ssh (MAC2-SSH build 50, tenant 1457, client 143.100.100.10363): DEM LaunchDaemon + pkg receipt present but process NOT running because tenant flag dem_agent_enabled is unset -- confirms the dormant-until-triggered baseline. This case needs a tenant with the flag ON to prove the trigger path.</t>
+          <t>NSClient's own startup/init sequence must be the sole trigger for DEM Agent start -- the agent does not auto-start on its own (note Q2b). REVISED after live verification (2026-10-08, tenant 1340/sys1340mac, build 54): confirmed via nsdebuglog.log lines 31-35 (stAgentSvc.cpp:72 "init m_demMgr", nsDemTaskMgr.cpp:131 "DEM init nsDemTaskMgr", stAgentSvc.cpp:97 "register DEM module callbacks") that NSClient initializes its OWN in-process DEM module (m_demMgr) at startup -- the old ch16 in-process module was NOT replaced, it coexists with the new standalone netskope-dem-agent process. No nsconfig.json flag named dem_agent_enabled was found in two separate live checks (tenant 1457 and 1340); the real enablement signal is the standalone agent's own nsdemconfig.json, fetched via its periodic poll_settings action.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Core decoupling requirement: DEM data collection AND config updates must continue when NSClient is disabled, as long as the endpoint can still reach events.goskope.com / dem-config.goskope.com (note lines 5-7). The OLD in-process DEM explicitly called demMgr.stop(true) as step 4 of service shutdown (ch03) -- the NEW standalone agent must NOT inherit that wiring.</t>
+          <t>Core decoupling requirement: DEM data collection AND config updates must continue when NSClient is disabled, as long as the endpoint can still reach events.goskope.com / dem-config.goskope.com (note lines 5-7). CAUTION after live evidence (2026-10-08, tenant 1340, build 54, nsdebuglog_dem_lines_tenant1340_build54_20261008.txt (local copy under C:\tmp\nplan-4237\)): this is NOT fully decoupled today. nsdebuglog.log line 3477 (tunnel.cpp:1336) shows NSClient's own tunnel actively steering the standalone netskope-dem-agent's app-probe traffic ("Tunneling flow from addr ... process: netskope-dem-agent to host: udemy.com ... to nsProxy"), repeating every ~5min (lines 3948, 4186, 4380, ... 6041). Only the Polaris event-receiver connection is explicitly bypassed from the tunnel (line 3502, demMgr.cpp:701 "DEM Bypassing connection to polaris event receiver... process netskope-dem-agent"). So TODAY: app-probe traffic appears tunnel-dependent, while GEF/Polaris event posting bypasses it. This case must verify EACH traffic class separately, not assume blanket independence.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>DEM Agent process terminates when NSClient is disabled.</t>
+          <t>DEM Agent process terminates when NSClient is disabled; OR (revised) app-probe traffic silently fails/stalls once the tunnel is unavailable (would mean the 'continues when disabled' requirement is unmet for that traffic class, even if the process itself survives) -- check both the process AND each traffic class's delivery, per the live evidence above.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Same decoupling invariant as SYS-4237-02 but scoped to tunnel-down rather than admin-disabled. The OLD in-process DEM explicitly stopped on onTunnelDisconnected (ch16: "data collection starts when a tunnel connects and stops when all tunnels disconnect"; ENG-593503 crash on this exact path). The new standalone agent must NOT replicate this tunnel-coupling -- it should use the Direct Internet Access path.</t>
+          <t>Same decoupling invariant as SYS-4237-02 but scoped to tunnel-down rather than admin-disabled. The OLD in-process DEM explicitly stopped on onTunnelDisconnected (ch16: "data collection starts when a tunnel connects and stops when all tunnels disconnect"; ENG-593503 crash on this exact path). CAUTION after live evidence (2026-10-08, tenant 1340, build 54): nsdebuglog.log line 3477 shows the standalone agent's app-probe traffic is ACTIVELY tunneled through NSClient ("process: netskope-dem-agent to host: udemy.com ... to nsProxy") -- if the tunnel goes down, this specific traffic class has no documented fallback path observed yet. Only the Polaris/GEF event path (line 3502) is confirmed to bypass the tunnel. This case must distinguish 'DEM process survives tunnel-down' from 'DEM app-probe traffic survives tunnel-down' -- live evidence suggests the latter may currently fail.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>DEM Agent treats tunnel-disconnect as a stop signal (reproduces the OLD coupling this refactor removes).</t>
+          <t>DEM Agent treats tunnel-disconnect as a stop signal (reproduces the OLD coupling this refactor removes) OR (revised, more likely per live evidence) the process survives but app-probe traffic silently stalls/fails because it has no direct-path fallback when NSClient's tunnel -- which it is currently routed through -- is down.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>ch16 ENG-637576: the OLD in-process DEM's config-rotation path could reset tenant_id to 0, causing the backend to reject ALL subsequent events. The standalone Agent now owns its OWN config-fetch path (dem-config.goskope.com) independent of NSClient's config rotation -- verify it does not inherit the same bug class.</t>
+          <t>ch16 ENG-637576: the OLD in-process DEM's config-rotation path could reset tenant_id to 0, causing the backend to reject ALL subsequent events. The standalone Agent now owns its OWN config-fetch path (dem-config.goskope.com) independent of NSClient's config rotation -- verify it does not inherit the same bug class. NOTE after live evidence (2026-10-08, tenant 1340, build 54): the OLD in-process m_demMgr/nsDemTaskMgr is confirmed STILL ACTIVE (nsdebuglog.log lines 31-35, 3502 and repeats) alongside the new standalone agent -- ENG-637576's ORIGINAL in-process code path is therefore still a live risk in its own right, not just a historical reference; this case should check tenant-ID integrity on BOTH the in-process module's GEF posts and the standalone agent's dem-config.goskope.com fetch.</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Gap-check SYSPLAN-4237 against 6 owner requirements, merge to 8 cases
Checked frequent process-liveness checks, service start/stop, crash-dump
scanning, max app-probe stress, disable/enable during active probing,
and stAgent<->DEM Agent probing handoff against the existing 9 cases.
Folded 5 of 6 gaps into the most thematically related existing case
(DEM-01/02/04); only the app-probe-count stress scenario needed a new
case (DEM-08). Net: merged DEM-05 into DEM-01 and DEM-07+DEM-08 into
DEM-06, landing at 8 cases total -- below the original 9.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,7 +481,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DEM Agent start is NSClient-triggered, not self-starting</t>
+          <t>DEM Agent lifecycle is NSClient-driven: start, clean stop, reboot</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -491,25 +491,26 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>DEM Agent must not self-start; NSClient's own init triggers it. Live-confirmed (live check tenant 1340/build 54, 2026-10-08): the OLD in-process m_demMgr still inits at NSClient startup alongside the new standalone agent (nsdebuglog.log lines 31-35) -- both exist, not a clean replacement.</t>
+          <t>DEM Agent must never self-start; only an NSClient start event (service start or post-reboot startup) triggers it, and a CLEAN NSClient service stop must not orphan it. Live-confirmed (live check tenant 1340/build 54, 2026-10-08): old in-process m_demMgr still inits at NSClient startup too (nsdebuglog.log lines 31-35).</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>1. Enroll NSClient, tenant with DEM enabled.
-2. Confirm DEM LaunchDaemon not yet started.
-3. Start NSClient.
-4. Poll for netskope-dem-agent process + err-log sync message, up to 60s.</t>
+          <t>1. Enroll NSClient, tenant with DEM enabled; confirm DEM LaunchDaemon not started.
+2. Start NSClient; poll for netskope-dem-agent process + sync log, up to 60s.
+3. Cleanly stop the NSClient service (not kill); verify DEM's resulting state is well-defined, not orphaned.
+4. Restart NSClient; confirm DEM comes back.
+5. Reboot VM; immediately confirm DEM NOT running; wait for NSClient startup; confirm DEM starts.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>netskope-dem-agent process appears within 60s of NSClient startup completing.</t>
+          <t>DEM only ever starts after an NSClient start event (service start or post-reboot); never autostarts; no orphan after a clean stop.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>DEM never starts (no monitoring data), or starts independently of NSClient (breaks the dependency contract).</t>
+          <t>Orphaned DEM running with no NSClient (stale monitoring data), or DEM never starting (monitoring gap).</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -531,7 +532,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DEM keeps working when NSClient is disabled</t>
+          <t>App-probe continuity across NSClient/DEM Agent availability (both directions)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -541,25 +542,24 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Core requirement: DEM must keep collecting/posting when NSClient is disabled. Live evidence (nsdebuglog.log lines 3477, 3502): app-probe traffic is tunneled THROUGH NSClient while Polaris/GEF posting bypasses it -- verify both paths, not just process survival.</t>
+          <t>Two continuity contracts in one case: (A) DEM keeps probing/posting when NSClient is disabled, and resumes cleanly when re-enabled; (B) when DEM Agent itself is unavailable, probing falls back to NSClient's own in-process path, and switches back once DEM is available again. Live evidence (nsdebuglog.log lines 3477, 3502): app-probe traffic is tunneled through NSClient while GEF/Polaris posting bypasses it -- verify per traffic class.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline: DEM running, posting events.
-2. Disable NSClient.
-3. Wait 2x DEM post interval.
-4. Check process alive, GEF/Polaris posting continues, AND app-probe traffic still succeeds.</t>
+          <t>1. Baseline: DEM Agent running, actively probing.
+2. (A) Disable NSClient mid-probe-cycle; verify DEM process + probing continues. Re-enable NSClient; verify probing resumes, no duplicate/missed cycle.
+3. (B) Disable/stop DEM Agent, NSClient stays enabled; verify probing switches to NSClient's own in-process path. Re-enable DEM Agent; verify probing switches back.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Process survives; GEF/Polaris posting continues; app-probe requests still complete.</t>
+          <t>No probing gap longer than one cycle in either direction; correct component probes at every stage; no duplicate data on handoff.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Monitoring data gap while NSClient is disabled -- defeats the decoupling goal.</t>
+          <t>Silent monitoring gap during normal admin ops (disable/re-enable, DEM maintenance) -- defeats the decoupling goal.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (lines 5-7) + ch03_service_lifecycle.md + nsdebuglog.log lines 3477/3502 (live check tenant 1340/build 54, 2026-10-08)</t>
+          <t>nplan-4237-note.txt (lines 5-7) + functional test plan (NS Client/DEM Agent sheets) (fallback case) + ch03_service_lifecycle.md + nsdebuglog.log lines 3477/3502</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DEM keeps working when NSClient tunnel is disconnected</t>
+          <t>DEM continues when NSClient tunnel disconnects, resumes on reconnect</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -591,24 +591,24 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Same as DEM-02 but tunnel-down, not admin-disabled. Old in-process DEM stopped on tunnel-disconnect (ch16); standalone agent's app-probe traffic is currently tunnel-routed (nsdebuglog.log lines 3477) and must not silently stall.</t>
+          <t>Distinct trigger from DEM-02 (network-layer, not admin action). Old in-process DEM stopped on tunnel-disconnect (ch16); standalone agent's app-probe traffic is tunnel-routed (same evidence as DEM-02, nsdebuglog.log lines 3477) and must not silently stall, then must resume cleanly on reconnect.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>1. Baseline running.
-2. Disconnect tunnel (block gateway), keep NSClient service enabled.
-3. Check DEM process + traffic path.</t>
+2. Disconnect tunnel (block gateway), keep NSClient service enabled; check DEM process + traffic path.
+3. Reconnect; verify probing/posting resumes without manual intervention.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>DEM process unaffected by tunnel state; app-probe traffic has a working path.</t>
+          <t>DEM process unaffected by tunnel state; probing has a working path or recovers immediately on reconnect.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>DEM data gap on every tunnel flap -- same impact class as DEM-02.</t>
+          <t>DEM data gap on every tunnel flap (a common event) -- same impact class as DEM-02.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NSClient crash/recovery does not orphan or duplicate DEM Agent</t>
+          <t>DEM Agent stays healthy and crash-free through NSClient crash/recovery</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -640,25 +640,25 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>NSClient crash+restart (ch03 TC-03-W04, 60s bound) must leave exactly one healthy DEM Agent instance.</t>
+          <t>Combines three health signals into one continuous-monitoring case: (1) DEM CPU/mem/handle sampled frequently throughout the run (sampler's dem_agent_enabled=True mode), (2) zero DEM Agent crash dumps appear in DiagnosticReports at any point, (3) NSClient crash+restart (ch03 TC-03-W04, 60s bound) leaves exactly one healthy DEM instance.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline both running.
-2. Force-kill NSClient process.
-3. Wait up to 60s for recovery.
-4. Count DEM Agent processes.</t>
+          <t>1. Start continuous resource sampler (CPU/mem/handle, 10s interval) for the whole test window.
+2. Baseline, then force-kill NSClient process; wait up to 60s for recovery.
+3. Count DEM Agent processes after recovery.
+4. At teardown, scan DiagnosticReports for any DEM Agent crash report.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Exactly 1 netskope-dem-agent process after recovery.</t>
+          <t>Sampler shows DEM alive throughout (no unexplained gaps); exactly 1 process after recovery; zero crash dumps.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Orphaned/duplicate DEM processes waste resources or double-post data.</t>
+          <t>Resource leak or crash goes undetected; orphaned/duplicate DEM processes after NSClient crash.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt + ch03_service_lifecycle.md (TC-03-W04)</t>
+          <t>nplan-4237-note.txt + ch03_service_lifecycle.md (TC-03-W04) + mac_system_info.py (crash_dumps/sample_tick)</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DEM Agent does not auto-start at boot; waits for NSClient</t>
+          <t>NSClient uninstall removes DEM Agent completely (known gap)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -690,26 +690,24 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Per owner note, DEM must NOT be a launchd auto-start item -- it must wait for NSClient's own startup to trigger it.</t>
+          <t>Owner note explicitly flags this as unhandled by the current (not-yet-merged) uninstaller -- expected-fail gap, tracked as the regression gate for when the fix lands.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline running.
-2. Reboot VM.
-3. Immediately check DEM process (expect absent).
-4. Wait for NSClient startup to finish.
-5. Re-check DEM process.</t>
+          <t>1. Baseline both installed.
+2. Uninstall NSClient normally.
+3. Check DEM process, LaunchDaemon, pkg receipt, and DEM data dir all removed.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>DEM absent right after boot; present only after NSClient finishes startup.</t>
+          <t>All DEM artifacts gone.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>RunAtLoad regression starts DEM before enrollment/config exists, or DEM never restarts post-reboot.</t>
+          <t>Orphaned DEM Agent keeps running/collecting after NSClient is gone.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -719,7 +717,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (Q2b) + ch03_service_lifecycle.md</t>
+          <t>nplan-4237-note.txt (Q2c + Answer 1b)</t>
         </is>
       </c>
     </row>
@@ -731,34 +729,34 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NSClient uninstall removes DEM Agent completely (known gap)</t>
+          <t>Upgrade independence between DEM Agent and NSClient (both directions)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DEM / Service Lifecycle (macOS)</t>
+          <t>DEM / Upgrade (macOS)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Owner note explicitly flags this as unhandled by the current (not-yet-merged) uninstaller -- expected-fail gap, tracked as the regression gate for when the fix lands.</t>
+          <t>Merges both upgrade-independence directions: (A) a DEM-only upgrade must not disrupt NSClient; (B) NSClient's own upgrade must not orphan/crash/duplicate DEM Agent.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline both installed.
-2. Uninstall NSClient normally.
-3. Check DEM process, LaunchDaemon, pkg receipt, and DEM data dir all removed.</t>
+          <t>1. Baseline both running.
+2. (A) Install a newer DEM Agent pkg only; monitor NSClient tunnel/service throughout -- must stay untouched.
+3. (B) Trigger NSClient auto-upgrade; monitor DEM Agent process through the upgrade+restart window.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>All DEM artifacts gone.</t>
+          <t>Neither upgrade disrupts the other component; DEM ends in exactly one healthy instance after (B).</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Orphaned DEM Agent keeps running/collecting after NSClient is gone.</t>
+          <t>A routine upgrade of either component causes unplanned disruption to the other, fleet-wide, every release.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -768,7 +766,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (Q2c + Answer 1b)</t>
+          <t>nplan-4237-note.txt (lines 15-17) + ch01_installation.md (PostInstallSuccess) + ch03_service_lifecycle.md</t>
         </is>
       </c>
     </row>
@@ -780,44 +778,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DEM-only upgrade has zero impact on NSClient</t>
+          <t>DEM Agent and in-process DEM module both keep correct tenant ID through config rotation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DEM / Upgrade (macOS)</t>
+          <t>DEM / Config Integrity (macOS)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Headline requirement: DEM software/config update must not disrupt the NSClient parent process or follow its release cadence.</t>
+          <t>ch16 ENG-637576: old in-process DEM could reset tenant_id to 0 during token rotation. Live-confirmed (nsdebuglog.log lines 31-35) the in-process module is STILL ACTIVE alongside the new agent -- both paths need checking, not just the new one.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline both running, note NSClient tunnel/service state.
-2. Install a newer DEM Agent pkg only.
-3. Monitor NSClient tunnel/service throughout.</t>
+          <t>1. Baseline both DEM Agent + in-process module posting successfully.
+2. Trigger NSClient secure-enrollment token rotation.
+3. Check tenant ID on BOTH the in-process GEF posts and the standalone agent's dem-config.goskope.com fetch.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>NSClient tunnel stays connected; NSClient service never restarts; DEM comes back on the new version.</t>
+          <t>Correct tenant ID on both paths throughout rotation.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>A routine DEM update causes unplanned NSClient disruption fleet-wide.</t>
+          <t>All DEM events rejected backend-side ("tenant ID does not match") -- reproduces ENG-637576 on two code paths instead of one.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ENG-637576 (analog, old architecture)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (lines 15-17) + ch01_installation.md + ch03_service_lifecycle.md</t>
+          <t>ch16_dem.md (ENG-637576) + nplan-4237-note.txt + nsdebuglog.log lines 31-35</t>
         </is>
       </c>
     </row>
@@ -829,34 +827,34 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NSClient auto-upgrade does not orphan or crash DEM Agent</t>
+          <t>App probe stress at maximum configured probe count</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DEM / Upgrade (macOS)</t>
+          <t>DEM / Scale (macOS)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Reverse direction of DEM-07 -- NSClient's own upgrade/restart cycle (ch01) must not leave DEM Agent orphaned, duplicated, or crashed.</t>
+          <t>NEW case. Configure the DEM network probe at its maximum supported count/frequency and verify stability -- ch16's RISK_LIMIT notes the OLD module's app-probe limit (default 10) silently drops probes beyond it; verify the standalone agent either enforces or clearly reports its own limit, and stays stable under max load.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline both running, DEM posting events.
-2. Trigger NSClient auto-upgrade.
-3. Monitor DEM process through the upgrade+restart window.</t>
+          <t>1. Configure the DEM network probe with the maximum supported number of app probes (per product limit) and minimum frequency.
+2. Run a sustained soak window with continuous CPU/mem/handle sampling (dem_agent_enabled=True).
+3. Verify every configured probe actually executes (not silently dropped) and NSClient's own resource usage stays within the existing health gate (CPU_SUSTAIN_PCT/MEM_GROWTH_MAX_MB).</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>DEM Agent ends in exactly one healthy instance; posting continues or resumes within a bounded restart window.</t>
+          <t>All configured probes execute; DEM Agent CPU/mem/handles stay bounded (no sustained growth); NSClient unaffected.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Silent monitoring gap or duplicate-process leak on every NSClient upgrade cycle, fleet-wide.</t>
+          <t>Probes silently dropped beyond a limit (stale/incomplete monitoring data), or resource exhaustion impacting NSClient at scale.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -866,56 +864,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt + ch01_installation.md (PostInstallSuccess) + ch03_service_lifecycle.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>DEM-09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DEM Agent and in-process DEM module both keep correct tenant ID through config rotation</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DEM / Config Integrity (macOS)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>ch16 ENG-637576: old in-process DEM could reset tenant_id to 0 during token rotation. Live-confirmed (nsdebuglog.log lines 31-35) the in-process module is STILL ACTIVE alongside the new agent -- both paths need checking, not just the new one.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>1. Baseline both DEM Agent + in-process module posting successfully.
-2. Trigger NSClient secure-enrollment token rotation.
-3. Check tenant ID on BOTH the in-process GEF posts and the standalone agent's dem-config.goskope.com fetch.</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Correct tenant ID on both paths throughout rotation.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>All DEM events rejected backend-side ("tenant ID does not match") -- reproduces ENG-637576 on two code paths instead of one.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>ENG-637576 (analog, old architecture)</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>ch16_dem.md (ENG-637576) + nplan-4237-note.txt + nsdebuglog.log lines 31-35</t>
+          <t>nplan-4237-note.txt + ch16_dem.md (RISK_LIMIT, app probe limit) + functional test plan (NS Client/DEM Agent sheets) (DEM Agent sheet, Long-duration stability)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine DEM-06: test real upgrade paths, not a standalone DEM pkg install
Owner correction: do not install a standalone DEM Agent pkg -- NSClient's
own installer bundle already carries dem_agent.pkg as a sibling component
(confirmed live in the STAgent.pkg Distribution XML). DEM-06 now exercises
NSClient's own auto-upgrade and a direct package reinstall, checking both
NSClient's and DEM Agent's status after each.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Upgrade independence between DEM Agent and NSClient (both directions)</t>
+          <t>NSClient upgrade (auto-upgrade or package reinstall) carries DEM Agent correctly</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -739,24 +739,24 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Merges both upgrade-independence directions: (A) a DEM-only upgrade must not disrupt NSClient; (B) NSClient's own upgrade must not orphan/crash/duplicate DEM Agent.</t>
+          <t>REVISED (owner): do NOT install a standalone DEM Agent pkg -- that is not the real upgrade path. NSClient's own installer bundle already carries dem_agent.pkg as a sibling component (confirmed live: the STAgent.pkg Distribution XML, client-feature-pipeline build 10363, lists pkg-ref id="dem_agent.pkg" version="2611.0.1.0" alongside com.netskope.STAgent.pkg). The real upgrade paths are NSClient's own auto-upgrade and a direct package reinstall (pkg upgrade) -- both must leave BOTH components correct and healthy afterward, with no separate DEM-only install step.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline both running.
-2. (A) Install a newer DEM Agent pkg only; monitor NSClient tunnel/service throughout -- must stay untouched.
-3. (B) Trigger NSClient auto-upgrade; monitor DEM Agent process through the upgrade+restart window.</t>
+          <t>1. Baseline: note NSClient version + DEM Agent version/process state.
+2. Trigger NSClient auto-upgrade to a newer build; after completion, check NSClient status (tunnel/service/version) AND DEM Agent status (process alive, version, LaunchDaemon) both reflect the new build.
+3. Separately, trigger a direct package upgrade (reinstall newer STAgent.pkg over the existing install); repeat the same dual status check.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Neither upgrade disrupts the other component; DEM ends in exactly one healthy instance after (B).</t>
+          <t>After EITHER upgrade path, NSClient is healthy on the new version AND DEM Agent is healthy on its bundled version -- no manual DEM reinstall needed.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>A routine upgrade of either component causes unplanned disruption to the other, fleet-wide, every release.</t>
+          <t>DEM Agent silently left on a stale version after an NSClient upgrade (undetected version drift), or the upgrade path breaks because it wrongly assumes DEM Agent needs separate handling.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (lines 15-17) + ch01_installation.md (PostInstallSuccess) + ch03_service_lifecycle.md</t>
+          <t>nplan-4237-note.txt (lines 15-17) + ch01_installation.md (PostInstallSuccess) + ch03_service_lifecycle.md + live pkg Distribution XML (client-feature-pipeline build 10363)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add DEM-09: DEM thread safety under sustained max-probe load (ENG-593503)
Owner-sourced case targeting ch16's ENG-593503 (DEM thread stack overrun
crashing stAgentSvc) on the OLD in-process DEM module -- confirmed not
covered by any of the 8 existing cases (DEM-08 stresses the standalone
agent's probe count, not the in-process module's thread/queue safety).
Back to 9 cases total.

Signed-off-by: Austin Cheng <acheng@netskope.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -868,6 +868,57 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DEM-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DEM thread does not overrun or crash NSClient under sustained max-probe load</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DEM / Thread Safety (macOS)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Owner-sourced case (external doc, exact origin not re-derived by this skill -- flagged honestly rather than inventing a citation). Targets ch16 ENG-593503: DEM thread stack overrun crashes stAgentSvc when DEM worker threads (nsTaskScheduler, up to 5 concurrent app-probe workers) are still active under load. This stresses the OLD in-process DEM module -- confirmed STILL ACTIVE per DEM-07 -- at sustained max probe load, distinct from DEM-08's standalone-agent probe-count test.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>1. Tenant: configure 50 DEM probes, all on 30s schedule.
+2. Run for 1 hour.
+3. Monitor DEM thread CPU and queue depth (nsTaskScheduler).
+4. Verify probes skip/back off when overloaded (backoff logged, not silently dropped).
+5. Verify no service crash (stAgentSvc), no missed config callbacks (onConfigUpdate cascade continues).</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Over the 1-hour run: DEM thread CPU/queue depth stays bounded (no runaway growth); overload triggers a logged backoff, not a crash; stAgentSvc never crashes; onConfigUpdate callback cascade never misses a cycle.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>ENG-593503-class crash (DEM thread stack overrun) under real-world probe load; or missed config callbacks corrupting tunnel/steering/FailClose state during the overload window.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ENG-593503</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ch16_dem.md (ENG-593503, DEM Thread Crash Flow + Cross-Flow Risk Matrix) + owner-provided case</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
spec(DEM-04): add direct DEM Agent kill robustness step
Live POC 2026-10-13 (tenant 1340, build 10329): killing netskope-dem-agent
directly (SIGKILL) is auto-relaunched by launchd within ~1s via the plist's
KeepAlive/SuccessfulExit:false -- reproducible across two independent
kills, new PID each time, no external trigger needed. DEM-04 is the only
case about DEM's own crash-resilience; its old steps only force-killed
NSClient, never the standalone DEM Agent process itself. Added as step 3,
renumbered the rest.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -647,13 +647,14 @@
         <is>
           <t>1. Start continuous resource sampler (CPU/mem/handle, 10s interval) for the whole test window.
 2. Baseline, then force-kill NSClient process; wait up to 60s for recovery.
-3. Count DEM Agent processes after recovery.
-4. At teardown, scan DiagnosticReports for any DEM Agent crash report.</t>
+3. Separately, force-kill the standalone DEM Agent process itself (netskope-dem-agent, SIGKILL) at least twice in a row; confirm launchd auto-relaunches it (KeepAlive/SuccessfulExit:false) within an expected bound each time -- validates DEM Agent crash-resilience independent of NSClient state (live-confirmed 2026-10-13, tenant 1340/build 10329: sub-1s auto-respawn, reproducible across 2 independent kills, new PID each time).
+4. Count DEM Agent processes after NSClient-crash recovery (step 2).
+5. At teardown, scan DiagnosticReports for any DEM Agent crash report.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Sampler shows DEM alive throughout (no unexplained gaps); exactly 1 process after recovery; zero crash dumps.</t>
+          <t>Sampler shows DEM alive throughout (no unexplained gaps); exactly 1 process after NSClient-crash recovery; a direct kill of the DEM Agent process itself is auto-relaunched by launchd within the expected bound every time (no manual/external action needed); zero crash dumps.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
spec(DEM-10): replace unobservable autostart race with static+causal proof
Live timing POC (2026-10-14): DEM registration completes ~20s after
kern.boottime; SSH is not reachable until 70-90s+ post-reboot. There is
no SSH-observable window where DEM is confirmed not-yet-running -- the
real startup finishes before any SSH probe can even run. Step 3 no
longer tries to catch that moment; it instead verifies
com.netskope.dem-agent.plist's RunAtLoad=false (static proof DEM never
self-starts via launchd independent of NSClient) plus that the
registration outcome line is timestamped after this boot's own
kern.boottime (causal proof it belongs to the current cycle, not a
stale leftover).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -943,15 +943,15 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>1. Baseline: DEM Agent running, registration confirmed.
-2. Reboot the VM (reuse POWER-04's reboot_vm_with_delay_mac).
-3. Immediately after SSH/NSClient recovery, before confirming full startup: check netskope-dem-agent is NOT running and NetskopeClientMacAppProxy's extension is not yet [activated enabled].
-4. Wait for NSClient's own startup (extension_loaded_mac confirms [activated enabled]).
+2. Reboot the VM (reuse POWER-04's reboot_vm_with_delay_mac); restage the mac probe script after SSH recovers (macOS wipes /tmp on every reboot, same gap POWER-04 already fixed).
+3. REVISED 2026-10-14 after live timing POC proved DEM registration completes ~20s post-boot while SSH is not reachable for 70-90s+ -- there is no SSH-observable window where DEM is confirmed not-yet-running post-reboot, so this step no longer races against that timing. Instead: (a) confirm com.netskope.dem-agent.plist's RunAtLoad is false (static proof DEM never self-starts via launchd independent of NSClient); (b) confirm the most recent "DEM module has been registered" outcome line in nsdebuglog.log is timestamped AFTER this reboot's own kern.boottime (causal proof this registration belongs to the current boot cycle, not a stale leftover line).
+4. Wait for NSClient's own startup (extension_loaded_mac confirms [activated enabled]) -- reuses POWER-04's own bound/poll-interval constants.
 5. Confirm DEM registration succeeds and netskope-dem-agent starts within a bounded time after NSClient's own startup.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DEM Agent never runs before NSClient's own post-reboot startup completes; DEM registration succeeds and the agent starts within a bounded time after that startup -- consistent behavior across a full OS reboot, not just a process-level restart.</t>
+          <t>DEM Agent's own LaunchDaemon is configured never to self-start independent of NSClient (RunAtLoad=false, statically verified); its registration after a reboot is attributable to that specific boot cycle (timestamped after kern.boottime); the agent starts within a bounded time of NSClient's own post-reboot startup. (Revised 2026-10-14: dropped the original "catch DEM not yet running immediately after SSH recovery" criterion -- live-proven mac-infeasible, the real startup completes before SSH is even reachable.)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
spec(DEM-02): drop fallback framing, only assert no missed probe cycle
Live research + a direct kill-disruption POC found the old in-process
module has no app-probe capability at all (nsDemConfig.cpp's
"AppProbes Cfg:" field is always empty, confirmed both at rest and
under sustained process disruption) -- there is no fallback path to
assert on. A DEM Agent restart instead triggers an extra probe cycle
immediately on respawn, never a gap. Per owner direction, duplicate
data is explicitly out of scope for this case's pass/fail -- only
confirm no probe cycle is ever missed, across (A) an NSClient
disable/enable toggle and (B) a DEM Agent process restart.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>App-probe continuity across NSClient/DEM Agent availability (both directions)</t>
+          <t>App-probe continuity across NSClient disable/enable and a DEM Agent restart</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -541,24 +541,24 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Two continuity contracts in one case: (A) DEM keeps probing/posting when NSClient is disabled, and resumes cleanly when re-enabled; (B) when DEM Agent itself is unavailable, probing falls back to NSClient's own in-process path, and switches back once DEM is available again. Live evidence (nsdebuglog.log lines 3477, 3502): app-probe traffic is tunneled through NSClient while GEF/Polaris posting bypasses it -- verify per traffic class.</t>
+          <t>REVISED 2026-10-14 after live research: (A) does the standalone DEM Agent keep running app probes uninterrupted while NSClient's tunnel is administratively disabled; (B) does a DEM Agent process restart (crash/kill) ever cause a MISSED probe cycle. Live research this session found the originally-assumed "falls back to NSClient's own in-process path" mechanism does NOT exist: the old in-process module (nsDemConfig.cpp) has an always-empty "AppProbes Cfg:" field -- confirmed both at rest and under a real, sustained process-kill disruption. A DEM Agent restart instead triggers an EXTRA probe cycle immediately on respawn, never a gap. Per owner direction, duplicate data is explicitly NOT a concern for this case -- only confirm no probe cycle is ever lost.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>1. Baseline: DEM Agent running, actively probing.
-2. (A) Disable NSClient mid-probe-cycle; verify DEM process + probing continues. Re-enable NSClient; verify probing resumes, no duplicate/missed cycle.
-3. (B) Disable/stop DEM Agent, NSClient stays enabled; verify probing switches to NSClient's own in-process path. Re-enable DEM Agent; verify probing switches back.</t>
+          <t>1. Baseline: DEM Agent running, actively probing on its configured frequency (confirm via dem-agent.err.log's "Running N app probe(s)" cadence).
+2. (A) Disable NSClient (client.disable()) mid-probe-cycle; confirm the DEM Agent process + probing continues uninterrupted (no cycle skipped) through at least one full probe interval while disabled. Re-enable NSClient (client.enable()); confirm probing continues with no missed cycle across the toggle.
+3. (B) Force-kill the DEM Agent process (netskope-dem-agent); confirm it auto-respawns (launchd KeepAlive) and that no probe cycle is missed across the disruption -- the gap between the probe cycle immediately before the kill and the next one logged (whether the regular-schedule cycle or an extra one triggered by the respawn) never exceeds the configured frequency plus a small margin.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>No probing gap longer than one cycle in either direction; correct component probes at every stage; no duplicate data on handoff.</t>
+          <t>No probe cycle is ever missed/lost across (A) an NSClient disable/enable toggle or (B) a DEM Agent process restart -- the maximum gap between consecutive probe cycles never exceeds the configured frequency plus margin. Duplicate/extra cycles are explicitly NOT a failure condition for this case.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Silent monitoring gap during normal admin ops (disable/re-enable, DEM maintenance) -- defeats the decoupling goal.</t>
+          <t>A genuinely missed probe cycle during normal admin ops (disable/re-enable) or a transient crash -- silent monitoring gap. (Duplicate data, while cosmetically redundant, is out of scope for this case's pass/fail, per owner direction.)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (lines 5-7) + functional test plan (NS Client/DEM Agent sheets) (fallback case) + ch03_service_lifecycle.md + nsdebuglog.log lines 3477/3502</t>
+          <t>nplan-4237-note.txt (lines 5-7) + ch03_service_lifecycle.md + 2026-10-14 live research (nsDemConfig.cpp AppProbes Cfg always empty; dem-agent.err.log run_app_probes/injector cadence; confirmed under live kill-disruption POC: respawns trigger an extra cycle, never a gap)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
spec(DEM-05): drop outdated known-gap framing, now a normal regression guard
Live-confirmed (build 89, tenant 1340/sys1340mac): a normal NSClient
uninstall genuinely removes all DEM artifacts (process, LaunchDaemon,
pkg receipt, data dir). The uninstaller fix this case was tracking as
expected-fail evidently landed (or never applied to this exact path) --
this is now a normal pass/fail regression guard, not an xfail-strict
case.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nplans/sysplan-nplan-4237.xlsx
+++ b/nplans/sysplan-nplan-4237.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NSClient uninstall removes DEM Agent completely (known gap)</t>
+          <t>NSClient uninstall removes DEM Agent completely</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Owner note explicitly flags this as unhandled by the current (not-yet-merged) uninstaller -- expected-fail gap, tracked as the regression gate for when the fix lands.</t>
+          <t>REVISED 2026-10-14: the original "known gap" framing (owner note, uninstaller not yet merged at the time) is now outdated -- live-confirmed (build 89, tenant 1340/sys1340mac) that a normal NSClient uninstall genuinely removes ALL DEM artifacts (process, LaunchDaemon, pkg receipt, data dir). This is now a normal regression guard against that gap recurring, not an expected-fail case.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -702,12 +702,12 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>All DEM artifacts gone.</t>
+          <t>All DEM artifacts (process, LaunchDaemon, pkg receipt, data dir) gone after a normal NSClient uninstall.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Orphaned DEM Agent keeps running/collecting after NSClient is gone.</t>
+          <t>Orphaned DEM Agent keeps running/collecting after NSClient is gone -- a regression of a previously-fixed gap.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>nplan-4237-note.txt (Q2c + Answer 1b)</t>
+          <t>nplan-4237-note.txt (Q2c + Answer 1b) + 2026-10-14 live confirmation (build 89, tenant 1340/sys1340mac, client-feature-pipeline 10329): pgrep/pkgutil/launchctl all clean post-uninstall -- the gap this case originally guarded as expected-fail no longer reproduces.</t>
         </is>
       </c>
     </row>

</xml_diff>